<commit_message>
voice recording is automatic and starts when game is resumed
</commit_message>
<xml_diff>
--- a/Python/subject_info.xlsx
+++ b/Python/subject_info.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UT\RAIIS\FBPerception\Python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{427BB826-5C8B-41ED-BDD9-9E4E6DE609E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7377851-EA1A-43D3-B3C4-09A44E8B82A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>ID</t>
   </si>
@@ -54,15 +54,9 @@
     <t>how often do you play joystick games(h per month)</t>
   </si>
   <si>
-    <t>Amir</t>
-  </si>
-  <si>
     <t>yes</t>
   </si>
   <si>
-    <t>male</t>
-  </si>
-  <si>
     <t>right</t>
   </si>
   <si>
@@ -73,6 +67,27 @@
   </si>
   <si>
     <t>Value</t>
+  </si>
+  <si>
+    <t>Cybersickness</t>
+  </si>
+  <si>
+    <t>Dobini</t>
+  </si>
+  <si>
+    <t>Which sense is superior</t>
+  </si>
+  <si>
+    <t>sleepness - tiredness (1-5)</t>
+  </si>
+  <si>
+    <t>Saba</t>
+  </si>
+  <si>
+    <t>female</t>
+  </si>
+  <si>
+    <t>vision</t>
   </si>
 </sst>
 </file>
@@ -399,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="43.77734375" customWidth="1"/>
@@ -408,10 +423,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -419,7 +434,7 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -427,7 +442,7 @@
         <v>0</v>
       </c>
       <c r="B3">
-        <v>9738</v>
+        <v>2541</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -435,7 +450,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -443,7 +458,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -451,7 +466,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -459,31 +474,63 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>8</v>
       </c>
-      <c r="B10">
-        <v>1</v>
+      <c r="B12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
first phase of experiment
</commit_message>
<xml_diff>
--- a/Python/subject_info.xlsx
+++ b/Python/subject_info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UT\RAIIS\FBPerception\Python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7377851-EA1A-43D3-B3C4-09A44E8B82A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74F250C5-B44B-4774-82E8-395B756E12AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,9 +57,6 @@
     <t>yes</t>
   </si>
   <si>
-    <t>right</t>
-  </si>
-  <si>
     <t>no</t>
   </si>
   <si>
@@ -81,13 +78,16 @@
     <t>sleepness - tiredness (1-5)</t>
   </si>
   <si>
-    <t>Saba</t>
-  </si>
-  <si>
-    <t>female</t>
-  </si>
-  <si>
-    <t>vision</t>
+    <t>male</t>
+  </si>
+  <si>
+    <t>Sadra</t>
+  </si>
+  <si>
+    <t>left</t>
+  </si>
+  <si>
+    <t>audio</t>
   </si>
 </sst>
 </file>
@@ -423,10 +423,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -442,7 +442,7 @@
         <v>0</v>
       </c>
       <c r="B3">
-        <v>2541</v>
+        <v>4177</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -458,7 +458,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -466,7 +466,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -474,15 +474,15 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -490,15 +490,15 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
@@ -519,15 +519,15 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
conducted experiment on first 3 subjects with this
</commit_message>
<xml_diff>
--- a/Python/subject_info.xlsx
+++ b/Python/subject_info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UT\RAIIS\FBPerception\Python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74F250C5-B44B-4774-82E8-395B756E12AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FF538B6-9A67-49B2-968A-E9064D85F88C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
   <si>
     <t>ID</t>
   </si>
@@ -78,16 +78,22 @@
     <t>sleepness - tiredness (1-5)</t>
   </si>
   <si>
+    <t>experiment type</t>
+  </si>
+  <si>
+    <t>Right</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Visual</t>
+  </si>
+  <si>
+    <t>Erfan</t>
+  </si>
+  <si>
     <t>male</t>
-  </si>
-  <si>
-    <t>Sadra</t>
-  </si>
-  <si>
-    <t>left</t>
-  </si>
-  <si>
-    <t>audio</t>
   </si>
 </sst>
 </file>
@@ -131,9 +137,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -422,114 +434,122 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="3">
+        <v>3914</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3">
-        <v>4177</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="3">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12">
-        <v>0</v>
-      </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="A14" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B14">
-        <v>4</v>
+      <c r="B14" s="3">
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="A15" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="3" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>